<commit_message>
Steering: agregar regla de siempre hacer push al final de cada ajuste
</commit_message>
<xml_diff>
--- a/outputs/IMAGENES_POR_ITT/itt_barrio_obrero/ITT_Barrio_Obrero.xlsx
+++ b/outputs/IMAGENES_POR_ITT/itt_barrio_obrero/ITT_Barrio_Obrero.xlsx
@@ -692,7 +692,7 @@
         <v>7</v>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" t="n">
         <v>80</v>
@@ -713,7 +713,7 @@
         <v>57.14</v>
       </c>
       <c r="O4" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="P4" t="n">
         <v>67</v>
@@ -722,7 +722,7 @@
         <v>92.20999999999999</v>
       </c>
       <c r="R4" t="n">
-        <v>63.75</v>
+        <v>60.41</v>
       </c>
       <c r="S4" t="n">
         <v>59.3</v>
@@ -731,7 +731,7 @@
         <v>54.9</v>
       </c>
       <c r="U4" t="n">
-        <v>69.8</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -804,6 +804,11 @@
           <t>periodo</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>es_proxy</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -838,6 +843,9 @@
           <t>2023-Q1</t>
         </is>
       </c>
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -872,6 +880,9 @@
           <t>2023-Q2</t>
         </is>
       </c>
+      <c r="K3" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -906,6 +917,9 @@
           <t>2023-Q3</t>
         </is>
       </c>
+      <c r="K4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -940,6 +954,9 @@
           <t>2023-Q4</t>
         </is>
       </c>
+      <c r="K5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -974,6 +991,9 @@
           <t>2024-Q1</t>
         </is>
       </c>
+      <c r="K6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1008,6 +1028,9 @@
           <t>2024-Q2</t>
         </is>
       </c>
+      <c r="K7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1042,6 +1065,9 @@
           <t>2024-Q3</t>
         </is>
       </c>
+      <c r="K8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1076,6 +1102,9 @@
           <t>2024-Q4</t>
         </is>
       </c>
+      <c r="K9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1110,6 +1139,9 @@
           <t>2025-Q1</t>
         </is>
       </c>
+      <c r="K10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1144,6 +1176,9 @@
           <t>2025-Q2</t>
         </is>
       </c>
+      <c r="K11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1178,6 +1213,9 @@
           <t>2025-Q3</t>
         </is>
       </c>
+      <c r="K12" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1205,12 +1243,52 @@
         <v>2</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>2025-Q4</t>
         </is>
+      </c>
+      <c r="K13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>44</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-Q1</t>
+        </is>
+      </c>
+      <c r="K14" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar Excel, notebook Av Cali y outputs Barrio Obrero
</commit_message>
<xml_diff>
--- a/outputs/IMAGENES_POR_ITT/itt_barrio_obrero/ITT_Barrio_Obrero.xlsx
+++ b/outputs/IMAGENES_POR_ITT/itt_barrio_obrero/ITT_Barrio_Obrero.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jorge\Desktop\Itt_repos_cali\outputs\IMAGENES_POR_ITT\itt_barrio_obrero\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FE2FB7-E1D2-4A6E-9B48-4FD0C95668C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D83147BA-FE22-4835-AC85-B4E4407B06AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="133">
   <si>
     <t>año</t>
   </si>
@@ -141,13 +141,292 @@
   </si>
   <si>
     <t>no</t>
+  </si>
+  <si>
+    <t>SEGUIMIENTO DATASETS — ITT CALI</t>
+  </si>
+  <si>
+    <t>Generado: Mayo 2026 | - = Sin datos | ** = Proxy</t>
+  </si>
+  <si>
+    <t>Zona</t>
+  </si>
+  <si>
+    <t>Area (m2)</t>
+  </si>
+  <si>
+    <t>Dimension ITT</t>
+  </si>
+  <si>
+    <t>Indicador</t>
+  </si>
+  <si>
+    <t>Peso</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Tipo Valor</t>
+  </si>
+  <si>
+    <t>Score/Valor</t>
+  </si>
+  <si>
+    <t>Periodo</t>
+  </si>
+  <si>
+    <t>Fuente</t>
+  </si>
+  <si>
+    <t>Formato</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t>Barrio Obrero</t>
+  </si>
+  <si>
+    <t>74,564</t>
+  </si>
+  <si>
+    <t>Seguridad</t>
+  </si>
+  <si>
+    <t>Homicidios</t>
+  </si>
+  <si>
+    <t>30%</t>
+  </si>
+  <si>
+    <t>COMPLETA</t>
+  </si>
+  <si>
+    <t>Real</t>
+  </si>
+  <si>
+    <t>Calculado</t>
+  </si>
+  <si>
+    <t>2023-2026 Q1</t>
+  </si>
+  <si>
+    <t>DATIC_homicidios_2023_2026T1_Barrio_O.geojson</t>
+  </si>
+  <si>
+    <t>GeoJSON</t>
+  </si>
+  <si>
+    <t>3 registros (2024-2025). Q2-Q4 2026 = -</t>
+  </si>
+  <si>
+    <t>Hurtos</t>
+  </si>
+  <si>
+    <t>DATIC_hurtos_2023_2026T1_Barrio_O.geojson</t>
+  </si>
+  <si>
+    <t>155 registros. Q2-Q4 2026 = -</t>
+  </si>
+  <si>
+    <t>Movilidad</t>
+  </si>
+  <si>
+    <t>Siniestralidad</t>
+  </si>
+  <si>
+    <t>25%</t>
+  </si>
+  <si>
+    <t>2023-2025</t>
+  </si>
+  <si>
+    <t>BD_SINIESTROS_2023_2025_COMUNA_BARRIO_OBRERO.geojson</t>
+  </si>
+  <si>
+    <t>15 registros. Sin datos 2026</t>
+  </si>
+  <si>
+    <t>Lesionados</t>
+  </si>
+  <si>
+    <t>BD_SINIESTROS (filtro Lesiones)</t>
+  </si>
+  <si>
+    <t>Filtro Tipo_Confi=Lesiones</t>
+  </si>
+  <si>
+    <t>Mortales</t>
+  </si>
+  <si>
+    <t>BD_SINIESTROS (filtro Mortal)</t>
+  </si>
+  <si>
+    <t>Filtro Tipo_Confi=Mortal</t>
+  </si>
+  <si>
+    <t>Entorno Urbano</t>
+  </si>
+  <si>
+    <t>Deficit Habitacional</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>PROXY</t>
+  </si>
+  <si>
+    <t>Proxy</t>
+  </si>
+  <si>
+    <t>39.2 (o recalculado)</t>
+  </si>
+  <si>
+    <t>2024</t>
+  </si>
+  <si>
+    <t>BD_DEFICIT_HABITACIONAL (Excel)</t>
+  </si>
+  <si>
+    <t>Excel</t>
+  </si>
+  <si>
+    <t>Proxy experimental Comuna 9</t>
+  </si>
+  <si>
+    <t>Educacion</t>
+  </si>
+  <si>
+    <t>Matricula</t>
+  </si>
+  <si>
+    <t>13%</t>
+  </si>
+  <si>
+    <t>Construccion</t>
+  </si>
+  <si>
+    <t>Proxy+Real</t>
+  </si>
+  <si>
+    <t>54.9 (23-25) / 31.5 (26)</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>geojson_educacion.zip</t>
+  </si>
+  <si>
+    <t>Proxy 54.9 para 2023-2025. Real 31.5 Q1 2026</t>
+  </si>
+  <si>
+    <t>Repitencia</t>
+  </si>
+  <si>
+    <t>Constante</t>
+  </si>
+  <si>
+    <t>6.82%</t>
+  </si>
+  <si>
+    <t>SIMAT 2026</t>
+  </si>
+  <si>
+    <t>Constante municipal</t>
+  </si>
+  <si>
+    <t>Est/Docente</t>
+  </si>
+  <si>
+    <t>24.64</t>
+  </si>
+  <si>
+    <t>Est/Equipo</t>
+  </si>
+  <si>
+    <t>22.3</t>
+  </si>
+  <si>
+    <t>03_Estudiantes_por_docente_y_equipo_2026.xlsx</t>
+  </si>
+  <si>
+    <t>Agregado sedes Comuna 9</t>
+  </si>
+  <si>
+    <t>Cohesion Social</t>
+  </si>
+  <si>
+    <t>VIF</t>
+  </si>
+  <si>
+    <t>12%</t>
+  </si>
+  <si>
+    <t>DATIC_violencia_intrafamiliar_2023_2026T1_Barrio_O.geojson</t>
+  </si>
+  <si>
+    <t>24 registros. Q2-Q4 2026 = -</t>
+  </si>
+  <si>
+    <t>Rinas</t>
+  </si>
+  <si>
+    <t>DATIC_comparendos_2023_2026T1_Barrio_O.geojson</t>
+  </si>
+  <si>
+    <t>Filtro startswith(RI). 374 reg total</t>
+  </si>
+  <si>
+    <t>Vulnerabilidad</t>
+  </si>
+  <si>
+    <t>54.1</t>
+  </si>
+  <si>
+    <t>Fijo</t>
+  </si>
+  <si>
+    <t>Pulmon de Oriente</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Score fijo heredado</t>
+  </si>
+  <si>
+    <t>RESUMEN POR ZONA</t>
+  </si>
+  <si>
+    <t>Area (ha)</t>
+  </si>
+  <si>
+    <t>7.46</t>
+  </si>
+  <si>
+    <t>Roosevelt</t>
+  </si>
+  <si>
+    <t>428,258</t>
+  </si>
+  <si>
+    <t>42.83</t>
+  </si>
+  <si>
+    <t>5,503,953</t>
+  </si>
+  <si>
+    <t>550.40</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,16 +434,57 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF666666"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1B4F8A"/>
+        <bgColor rgb="FF1B4F8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
+        <bgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3E0"/>
+        <bgColor rgb="FFFFF3E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE3F2FD"/>
+        <bgColor rgb="FFE3F2FD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -172,12 +492,56 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,10 +844,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:Y24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="17" max="17" width="14.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -551,7 +918,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2023</v>
       </c>
@@ -619,7 +986,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2024</v>
       </c>
@@ -687,7 +1054,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2025</v>
       </c>
@@ -755,7 +1122,655 @@
         <v>22</v>
       </c>
     </row>
+    <row r="9" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="Q9" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="R9" s="2"/>
+      <c r="S9" s="2"/>
+      <c r="T9" s="2"/>
+      <c r="U9" s="2"/>
+      <c r="V9" s="2"/>
+      <c r="W9" s="2"/>
+      <c r="X9" s="2"/>
+      <c r="Y9" s="2"/>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="Q10" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="R10" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="S10" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="T10" s="2"/>
+      <c r="U10" s="2"/>
+      <c r="V10" s="2"/>
+      <c r="W10" s="2"/>
+      <c r="X10" s="2"/>
+      <c r="Y10" s="2"/>
+    </row>
+    <row r="11" spans="1:25" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q11" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="R11" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="S11" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="2"/>
+      <c r="W11" s="2"/>
+      <c r="X11" s="2"/>
+      <c r="Y11" s="2"/>
+    </row>
+    <row r="12" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q12" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="R12" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="S12" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="T12" s="2"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="2"/>
+      <c r="W12" s="2"/>
+      <c r="X12" s="2"/>
+      <c r="Y12" s="2"/>
+    </row>
+    <row r="13" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q13" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="R13" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="S13" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="T13" s="2"/>
+      <c r="U13" s="2"/>
+      <c r="V13" s="2"/>
+      <c r="W13" s="2"/>
+      <c r="X13" s="2"/>
+      <c r="Y13" s="2"/>
+    </row>
+    <row r="14" spans="1:25" ht="120" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q14" s="10"/>
+      <c r="R14" s="10"/>
+      <c r="S14" s="10"/>
+      <c r="T14" s="10"/>
+      <c r="U14" s="10"/>
+      <c r="V14" s="10"/>
+      <c r="W14" s="10"/>
+      <c r="X14" s="10"/>
+      <c r="Y14" s="10"/>
+    </row>
+    <row r="15" spans="1:25" ht="75" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" ht="60" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="J24" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="K24" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="L24" s="5" t="s">
+        <v>124</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A9:L9"/>
+    <mergeCell ref="A10:L10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>